<commit_message>
[fix] pin position in power cable
</commit_message>
<xml_diff>
--- a/elec_gripette_hub_and_dyn/cables/CAB01206_Gripette_internal_power_cable.xlsx
+++ b/elec_gripette_hub_and_dyn/cables/CAB01206_Gripette_internal_power_cable.xlsx
@@ -630,9 +630,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>196200</xdr:colOff>
+      <xdr:colOff>195840</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>34560</xdr:rowOff>
+      <xdr:rowOff>34200</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -646,7 +646,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3809880" y="0"/>
-          <a:ext cx="1296720" cy="470160"/>
+          <a:ext cx="1296360" cy="469800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -671,10 +671,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>718560</xdr:colOff>
-      <xdr:row>58</xdr:row>
-      <xdr:rowOff>95040</xdr:rowOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>467640</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>160200</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -688,7 +688,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="13723200" cy="9523440"/>
+          <a:ext cx="14285160" cy="9913680"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>